<commit_message>
feat(mop): support merchant code KOC material packs
</commit_message>
<xml_diff>
--- a/adapters/mop-ops-assistant/templates/kol-material-img2video-template.xlsx
+++ b/adapters/mop-ops-assistant/templates/kol-material-img2video-template.xlsx
@@ -11,8 +11,8 @@
     <sheet name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'填写任务'!$A$1:$F$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段说明'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'填写任务'!$A$1:$G$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段说明'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,16 +462,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="68" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="86" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="68" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="86" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -482,30 +483,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>商家编码</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>素材图片</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>素材张数</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>比例</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>提示词</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>填写说明</t>
         </is>
@@ -517,22 +523,27 @@
           <t>728857154429</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="n">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>46X096070266</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>3:4</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>素材图片可留空：在 UI 选择素材根目录后读取 商品ID/01.jpg 到 03.jpg</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>素材图片可留空：在 UI 选择业务图包根目录后，按商家编码自动读取 图片/主图/达人 下的前 3 张</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>现在脚本按千牛页面的“选商品 + 图片生成展示视频”逻辑提交，不再选择或指定模板。
 素材图片不是必填；如果留空，请在运行界面选择“素材根目录”或“手动选择素材图片”。</t>
@@ -547,29 +558,36 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>564231A5355Z</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>/Users/you/Desktop/KOL素材/741042967594/01.jpg;/Users/you/Desktop/KOL素材/741042967594/02.jpg</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>3:4</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>突出版型和面料质感</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>示例：直接填写多张素材图片路径</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>素材根目录约定：素材根目录/商品ID/01.jpg、02.jpg、03.jpg。
-手动多选命名约定：商品ID_01.jpg，或父文件夹名为商品ID。
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>商品ID和商家编码二选一必填；商品ID为空时，脚本会自动按商家编码去千牛“我的商品”解析商品ID。
+业务图包约定：素材根目录/含商家编码的商品文件夹/图片/主图/达人/图片；顶层目录可用 + 关联多个商家编码。
+未匹配业务图包时，兼容旧规则：素材根目录/商品ID或商家编码/01.jpg、02.jpg、03.jpg。
+手动多选命名约定：商品ID_01.jpg 或 商家编码_01.jpg，或父文件夹名为商品ID/商家编码。
 素材图片列支持本地绝对路径或 http(s) 图片 URL；多张可用换行、分号、竖线或空格分隔。</t>
         </is>
       </c>
@@ -582,6 +600,7 @@
       <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="n"/>
@@ -591,6 +610,7 @@
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -600,6 +620,7 @@
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -609,6 +630,7 @@
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -618,6 +640,7 @@
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -627,6 +650,7 @@
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -636,6 +660,7 @@
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -645,6 +670,7 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="2" t="n"/>
@@ -654,6 +680,7 @@
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="2" t="n"/>
@@ -663,6 +690,7 @@
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="n"/>
@@ -672,6 +700,7 @@
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="2" t="n"/>
@@ -681,6 +710,7 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="n"/>
@@ -690,6 +720,7 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="2" t="n"/>
@@ -699,6 +730,7 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="2" t="n"/>
@@ -708,6 +740,7 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="2" t="n"/>
@@ -717,6 +750,7 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="2" t="n"/>
@@ -726,6 +760,7 @@
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="2" t="n"/>
@@ -735,6 +770,7 @@
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="2" t="n"/>
@@ -744,6 +780,7 @@
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2" t="n"/>
@@ -753,6 +790,7 @@
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="2" t="n"/>
@@ -762,6 +800,7 @@
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="2" t="n"/>
@@ -771,6 +810,7 @@
       <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="2" t="n"/>
@@ -780,6 +820,7 @@
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="2" t="n"/>
@@ -789,6 +830,7 @@
       <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="2" t="n"/>
@@ -798,6 +840,7 @@
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="2" t="n"/>
@@ -807,6 +850,7 @@
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="2" t="n"/>
@@ -816,11 +860,12 @@
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F30"/>
+  <autoFilter ref="A1:G30"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"3:4,1:1,9:16,16:9"</formula1>
     </dataValidation>
   </dataValidations>
@@ -834,7 +879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -873,12 +918,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>二选一</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>千牛/淘宝商品 ID；脚本会用该 ID 搜索商品，并把素材图片作为该商品的展示视频素材提交</t>
+          <t>千牛/淘宝商品 ID；有值时优先使用。为空但填写商家编码时，脚本会自动解析商品ID</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -890,29 +935,29 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>素材图片</t>
+          <t>商家编码</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>二选一</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>本地绝对路径或 http(s) 图片 URL；多张用换行、分号、竖线或空格分隔。也可以留空，改在 UI 选择素材根目录或手动多选素材图片</t>
+          <t>店铺内部商家编码；商品ID为空时，脚本会去千牛“我的商品”按商家编码搜索并取回商品ID</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>/Users/you/Desktop/KOL素材/728857154429/01.jpg;/Users/you/Desktop/KOL素材/728857154429/02.jpg</t>
+          <t>46X096070266</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>素材张数</t>
+          <t>素材图片</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -922,19 +967,19 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>素材图片为空且填写了“素材根目录”时生效；默认读取 素材根目录/商品ID/01.jpg 到 NN.jpg</t>
+          <t>本地绝对路径或 http(s) 图片 URL；多张用换行、分号、竖线或空格分隔。也可以留空，改在 UI 选择素材根目录或手动多选素材图片</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>/Users/you/Desktop/KOL素材/728857154429/01.jpg;/Users/you/Desktop/KOL素材/728857154429/02.jpg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>比例</t>
+          <t>素材张数</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -944,19 +989,19 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>展示视频生成比例；为空使用运行界面的默认比例</t>
+          <t>素材图片为空且填写了“素材根目录”时生效；业务图包按顺序取 图片/主图/达人 下前 N 张；旧规则读取 01.jpg 到 NN.jpg</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>提示词</t>
+          <t>比例</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -966,19 +1011,19 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>传给每张图片的生成提示；为空则不传</t>
+          <t>展示视频生成比例；为空使用运行界面的默认比例</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>突出商品版型和面料质感</t>
+          <t>3:4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>提示词</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -988,61 +1033,83 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>原样带到结果里，便于人工追踪</t>
+          <t>传给每张图片的生成提示；为空则不传</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>第一批 KOL 素材</t>
+          <t>突出商品版型和面料质感</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>素材包摆放</t>
+          <t>备注</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>建议</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>使用素材根目录时按“素材根目录/商品ID/01.jpg、02.jpg、03.jpg”摆放；扩展名固定为 jpg；png/jpeg/webp 请写入素材图片列或手动多选</t>
+          <t>原样带到结果里，便于人工追踪</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>/Users/you/Desktop/KOL素材/728857154429/01.jpg</t>
+          <t>第一批 KOL 素材</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>素材包摆放</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>推荐业务图包：素材根目录/MOP655137Z4106Z+656939D1213Y/图片/主图/达人/图片；顶层目录可用 + 关联多个商家编码；脚本只取主图图片，忽略视频和买家秀</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>/Users/you/Desktop/KOL素材/MOP655137Z4106Z+656939D1213Y/图片/主图/AHOYECHO/xxx.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>手动多选命名</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>建议</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>使用“手动选择素材图片”时，文件名以商品ID开头或父文件夹为商品ID；脚本会按商品ID自动归组</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>728857154429_01.jpg 或 728857154429/01.jpg</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>使用“手动选择素材图片”时，文件名以商品ID/商家编码开头或父文件夹为商品ID/商家编码；脚本会自动归组</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>46X096070266_01.jpg 或 46X096070266/01.jpg</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(mop): assign creator packages for duplicate merchant rows
</commit_message>
<xml_diff>
--- a/adapters/mop-ops-assistant/templates/kol-material-img2video-template.xlsx
+++ b/adapters/mop-ops-assistant/templates/kol-material-img2video-template.xlsx
@@ -11,8 +11,8 @@
     <sheet name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'填写任务'!$A$1:$G$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段说明'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'填写任务'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段说明'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,17 +462,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="68" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="86" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
+    <col width="92" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -488,30 +489,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>达人</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>素材图片</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>素材张数</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>比例</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>提示词</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>填写说明</t>
         </is>
@@ -529,28 +535,29 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>3:4</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>素材图片可留空：在 UI 选择业务图包根目录后，按商家编码自动读取 图片/主图/达人 下的前 3 张</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>素材图片可留空：同款单行会按主图下每个达人文件夹各生成一条；同款多行会按行顺序分配达人包，也可填写达人精确指定</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>现在脚本按千牛页面的“选商品 + 图片生成展示视频”逻辑提交，不再选择或指定模板。
 素材图片不是必填；如果留空，请在运行界面选择“素材根目录”或“手动选择素材图片”。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="72" customHeight="1">
+    <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>741042967594</t>
@@ -563,29 +570,37 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>达人A</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>/Users/you/Desktop/KOL素材/741042967594/01.jpg;/Users/you/Desktop/KOL素材/741042967594/02.jpg</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>3:4</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>突出版型和面料质感</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>示例：直接填写多张素材图片路径</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>商品ID和商家编码二选一必填；商品ID为空时，脚本会自动按商家编码去千牛“我的商品”解析商品ID。
 业务图包约定：素材根目录/含商家编码的商品文件夹/图片/主图/达人/图片；顶层目录可用 + 关联多个商家编码。
+如果同款只填一行，脚本会按主图下的每个达人文件夹拆成多条内容，每个达人文件夹各取前 N 张素材。
+如果同款在表格里填写多行，脚本会按行顺序分配达人图片包；每行自己的比例、提示词、备注会保留。
+可选填写“达人”列精确指定达人文件夹名。
 未匹配业务图包时，兼容旧规则：素材根目录/商品ID或商家编码/01.jpg、02.jpg、03.jpg。
 手动多选命名约定：商品ID_01.jpg 或 商家编码_01.jpg，或父文件夹名为商品ID/商家编码。
 素材图片列支持本地绝对路径或 http(s) 图片 URL；多张可用换行、分号、竖线或空格分隔。</t>
@@ -601,6 +616,7 @@
       <c r="F4" s="2" t="n"/>
       <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="n"/>
@@ -611,6 +627,7 @@
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="n"/>
@@ -621,6 +638,7 @@
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="2" t="n"/>
@@ -631,6 +649,7 @@
       <c r="F7" s="2" t="n"/>
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="n"/>
@@ -641,6 +660,7 @@
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="n"/>
@@ -651,6 +671,7 @@
       <c r="F9" s="2" t="n"/>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="2" t="n"/>
@@ -661,6 +682,7 @@
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="2" t="n"/>
@@ -671,6 +693,7 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="2" t="n"/>
@@ -681,6 +704,7 @@
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="2" t="n"/>
@@ -691,6 +715,7 @@
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="2" t="n"/>
@@ -701,6 +726,7 @@
       <c r="F14" s="2" t="n"/>
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="2" t="n"/>
@@ -711,6 +737,7 @@
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="n"/>
@@ -721,6 +748,7 @@
       <c r="F16" s="2" t="n"/>
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="2" t="n"/>
@@ -731,6 +759,7 @@
       <c r="F17" s="2" t="n"/>
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="2" t="n"/>
@@ -741,6 +770,7 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="2" t="n"/>
@@ -751,6 +781,7 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="2" t="n"/>
@@ -761,6 +792,7 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="2" t="n"/>
@@ -771,6 +803,7 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="2" t="n"/>
@@ -781,6 +814,7 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2" t="n"/>
@@ -791,6 +825,7 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="2" t="n"/>
@@ -801,6 +836,7 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="2" t="n"/>
@@ -811,6 +847,7 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="2" t="n"/>
@@ -821,6 +858,7 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="2" t="n"/>
@@ -831,6 +869,7 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="2" t="n"/>
@@ -841,6 +880,7 @@
       <c r="F28" s="2" t="n"/>
       <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="2" t="n"/>
@@ -851,6 +891,7 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="2" t="n"/>
@@ -861,11 +902,12 @@
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G30"/>
+  <autoFilter ref="A1:H30"/>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"3:4,1:1,9:16,16:9"</formula1>
     </dataValidation>
   </dataValidations>
@@ -879,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -957,7 +999,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>素材图片</t>
+          <t>达人</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -967,19 +1009,19 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>本地绝对路径或 http(s) 图片 URL；多张用换行、分号、竖线或空格分隔。也可以留空，改在 UI 选择素材根目录或手动多选素材图片</t>
+          <t>填写业务图包主图下的达人文件夹名时，会精确使用该达人图片包；不填时，单行同款会展开全部达人，多行重复同款会按行顺序分配达人包</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>/Users/you/Desktop/KOL素材/728857154429/01.jpg;/Users/you/Desktop/KOL素材/728857154429/02.jpg</t>
+          <t>AHOYECHO</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>素材张数</t>
+          <t>素材图片</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -989,19 +1031,19 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>素材图片为空且填写了“素材根目录”时生效；业务图包按顺序取 图片/主图/达人 下前 N 张；旧规则读取 01.jpg 到 NN.jpg</t>
+          <t>本地绝对路径或 http(s) 图片 URL；多张用换行、分号、竖线或空格分隔。也可以留空，改在 UI 选择素材根目录或手动多选素材图片</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>/Users/you/Desktop/KOL素材/728857154429/01.jpg;/Users/you/Desktop/KOL素材/728857154429/02.jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>比例</t>
+          <t>素材张数</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1011,19 +1053,19 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>展示视频生成比例；为空使用运行界面的默认比例</t>
+          <t>素材图片为空且填写了“素材根目录”时生效；单行同款展开全部达人，多行重复同款按行顺序分配达人包；每条取对应达人前 N 张；旧规则读取 01.jpg 到 NN.jpg</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3:4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>提示词</t>
+          <t>比例</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1033,19 +1075,19 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>传给每张图片的生成提示；为空则不传</t>
+          <t>展示视频生成比例；为空使用运行界面的默认比例</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>突出商品版型和面料质感</t>
+          <t>3:4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>提示词</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1055,61 +1097,83 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>原样带到结果里，便于人工追踪</t>
+          <t>传给每张图片的生成提示；为空则不传</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>第一批 KOL 素材</t>
+          <t>突出商品版型和面料质感</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>素材包摆放</t>
+          <t>备注</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>建议</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>推荐业务图包：素材根目录/MOP655137Z4106Z+656939D1213Y/图片/主图/达人/图片；顶层目录可用 + 关联多个商家编码；脚本只取主图图片，忽略视频和买家秀</t>
+          <t>原样带到结果里，便于人工追踪</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>/Users/you/Desktop/KOL素材/MOP655137Z4106Z+656939D1213Y/图片/主图/AHOYECHO/xxx.jpg</t>
+          <t>第一批 KOL 素材</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>素材包摆放</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>建议</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>推荐业务图包：素材根目录/MOP655137Z4106Z+656939D1213Y/图片/主图/达人/图片；顶层目录可用 + 关联多个商家编码；脚本只取主图图片，忽略视频和买家秀；多个达人文件夹可自动展开或按重复行分配</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>/Users/you/Desktop/KOL素材/MOP655137Z4106Z+656939D1213Y/图片/主图/AHOYECHO/xxx.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>手动多选命名</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>建议</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>使用“手动选择素材图片”时，文件名以商品ID/商家编码开头或父文件夹为商品ID/商家编码；脚本会自动归组</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>46X096070266_01.jpg 或 46X096070266/01.jpg</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>